<commit_message>
fix: error 500 ATS analyze - fix ATSAnalyzer call & add _get_company helper
</commit_message>
<xml_diff>
--- a/media/testing jabatan dan departemen.xlsx
+++ b/media/testing jabatan dan departemen.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project Pyton\HRIS-Updated-v3\hris_output\static\images\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project Pyton\BackUp-HRIS-SMARTDESK -3 - Deploy\media\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B5EE81FA-50F9-415C-8778-78D1A21BE7F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{790B308E-2E83-4F29-9B99-96719D8BB7F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C055B750-2FAD-4A97-A9C6-0F998466A184}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="261">
   <si>
     <t>KTT</t>
   </si>
@@ -457,6 +457,366 @@
   </si>
   <si>
     <t>Manajer Umum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Helper Kitchen Crew, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Safetyman, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Helper Waterman, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Helper Mechanic, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Crew Nursery Garden, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ABK Kapal, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Office Girl, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cleaning Service, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Personil Pemadam, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Carpenter, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Welder, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Technician, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Mechanic, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Electric Officer, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Operator Genset, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Driver LV/Truck, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Operator ADT, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Operator Dozer, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Operator DT, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Operator Excavator, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Operator Grader, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Operator Loader, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Admin Lab Preparasi, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Analis Lab, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Operator Crusher, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Operator Weighbridge, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Store Keeper, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Packer, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Security, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Tukang Kebun, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Clerk Admin HSE, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Clerk Admin Mechanic, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Clerk Admin GA, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Clerk Admin Civil, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Clerk Admin Legal, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Checker Rental, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Checker Admin Logistic, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Admin GA, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Admin Lab, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Safety Officer, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    HSE Officer, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    IT Officer, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    GS Officer, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Finance Officer, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Purchasing Officer, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Legal Officer, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Surveyor Site, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Interpreter Site, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Interpreter/Admin Site, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Admin cum Translator, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    GS Officer Cum Translator, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Admin Logistic Cum Translator, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    HR Admin Cum Translator, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Admin GA Cum Translator, Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Mekanik Senior, Senior Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Electric Officer Senior, Senior Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Operator Senior, Senior Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Foreman Cum Humas, Senior Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Foreman Mechanic, Senior Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Foreman Safety, Senior Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Foreman Mechanic AC, Senior Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Foreman HE Mechanic, Senior Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Foreman Electric, Senior Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Foreman Civil, Senior Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Junior Leader Safeguard, Senior Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Leader, Senior Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Chief Safeguard, Senior Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Senior Leader, Senior Staff,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Junior Supervisor Workshop, Junior Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Junior Supervisor Logistik, Junior Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Junior Supervisor GA, Junior Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Junior Foreman, Junior Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Koordinator Lapangan, Junior Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Koordinator Shift Mekanik, Junior Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Supervisor GA, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Supervisor Logistik, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Supervisor HSE, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Supervisor Civil, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Supervisor Mekanik, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Supervisor Electric, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Supervisor IT, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Supervisor HR, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Supervisor Keuangan, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Supervisor Pembelian, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Supervisor Legal, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Supervisor Umum, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Staff KTT, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    KTT, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Maintenance Coordinator, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Production Coordinator, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    HR Senior Officer, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    IT Assistant Manager, Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Senior Supervisor Workshop, Senior Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Senior Supervisor Logistik, Senior Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Senior Supervisor Civil, Senior Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Senior Supervisor Tambang, Senior Supervisor,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Assistant Manager, Junior Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Asisten Manajer HSE, Junior Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Asisten Manajer GA, Junior Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Asisten Manajer HR, Junior Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Asisten Manajer Keuangan, Junior Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Asisten Manajer Legal, Junior Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Asisten Manajer IT, Junior Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Asisten Manajer Logistik, Junior Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Asisten Manajer Produksi, Junior Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Asisten Manajer Pemeliharaan, Junior Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Manager CHP, Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Manager HR Advisor, Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Manajer HSE, Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Manajer GA, Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Manajer Logistik, Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Manajer Keuangan, Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Manajer Pembelian, Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Manajer Legal, Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Manajer IT, Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Manajer Tambang, Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Manajer Produksi, Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Manajer Pemeliharaan, Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Manajer Civil, Manager,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Manajer Umum, Manager,</t>
   </si>
 </sst>
 </file>
@@ -840,685 +1200,1046 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA1082FC-859B-40E0-8D48-C60F0B5F5D80}">
-  <dimension ref="A1:D125"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="46" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D5" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D6" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F6" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>75</v>
       </c>
       <c r="D7" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F7" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D8" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F8" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D9" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F9" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D10" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F10" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D11" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D12" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F12" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
       <c r="D13" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F13" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D14" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F14" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D15" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F15" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>15</v>
       </c>
       <c r="D16" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F16" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D17" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F17" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F18" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F19" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F20" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F21" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F22" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D23" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F23" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D24" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F24" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D25" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F25" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F26" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D27" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F27" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D28" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F28" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D29" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F29" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D30" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F30" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D31" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F31" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="33" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F32" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="33" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D33" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="34" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F33" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="34" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D34" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="35" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F34" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="35" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D35" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="36" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F35" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="36" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D36" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="37" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F36" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="37" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D37" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="38" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F37" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="38" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D38" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="39" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F38" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="39" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D39" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="40" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F39" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="40" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D40" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="41" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F40" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="41" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D41" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="42" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F41" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="42" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D42" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="43" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F42" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="43" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D43" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="44" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F43" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="44" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D44" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="45" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F44" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="45" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D45" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="46" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F45" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="46" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D46" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="47" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F46" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="47" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D47" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="48" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F47" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="48" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D48" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="49" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F48" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="49" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D49" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="50" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F49" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="50" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D50" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="51" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F50" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="51" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D51" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="52" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F51" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="52" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D52" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="53" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F52" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="53" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D53" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="54" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F53" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="54" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D54" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="55" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F54" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="55" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D55" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="56" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F55" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="56" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D56" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="57" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F56" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="57" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D57" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="58" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F57" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="58" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D58" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="59" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F58" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="59" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D59" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="60" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F59" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="60" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D60" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="61" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F60" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="61" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D61" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="62" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F61" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="62" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D62" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="63" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F62" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="63" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D63" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="64" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F63" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="64" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D64" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="65" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F64" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="65" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D65" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="66" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F65" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="66" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D66" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="67" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F66" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="67" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D67" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="68" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F67" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="68" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D68" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="69" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F68" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="69" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D69" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="70" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F69" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="70" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D70" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="71" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F70" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="71" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D71" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="72" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F71" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="72" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D72" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="73" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F72" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="73" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D73" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="74" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F73" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="74" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D74" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="75" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F74" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="75" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D75" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="76" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F75" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="76" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D76" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="77" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F76" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="77" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D77" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="78" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F77" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="78" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D78" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="79" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F78" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="79" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D79" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="80" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F79" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="80" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D80" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="81" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F80" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="81" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D81" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="82" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F81" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="82" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D82" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="83" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F82" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="83" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D83" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="84" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F83" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="84" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D84" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="85" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F84" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="85" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D85" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="86" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F85" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="86" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D86" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="87" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F86" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="87" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D87" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="88" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F87" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="88" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D88" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="89" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F88" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="89" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D89" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="90" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F89" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="90" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D90" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="91" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F90" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="91" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D91" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="92" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F91" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="92" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D92" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="93" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F92" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="93" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D93" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="94" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F93" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="94" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D94" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="95" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F94" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="95" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D95" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="96" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F95" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="96" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D96" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="97" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F96" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="97" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D97" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="98" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F97" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="98" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D98" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="99" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F98" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="99" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D99" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="100" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F99" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="100" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D100" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="101" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F100" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="101" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D101" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="102" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F101" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="102" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D102" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="103" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F102" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="103" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D103" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="104" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F103" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="104" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D104" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="105" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F104" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="105" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D105" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="106" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F105" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="106" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D106" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="107" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F106" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="107" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D107" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="108" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F107" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="108" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D108" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="109" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F108" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="109" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D109" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="110" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F109" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="110" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D110" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="111" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F110" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="111" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D111" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="112" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F111" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="112" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D112" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="113" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F112" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="113" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D113" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="114" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F113" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="114" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D114" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="115" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F114" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="115" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D115" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="116" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F115" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="116" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D116" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="117" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F116" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="117" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D117" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="118" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F117" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="118" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D118" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="119" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F118" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="119" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D119" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="120" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F119" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="120" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D120" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="121" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="F120" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="121" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D121" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="122" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="122" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D122" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="123" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="123" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D123" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="124" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="124" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D124" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="125" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="125" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D125" t="s">
         <v>140</v>
       </c>

</xml_diff>

<commit_message>
feat: migrate storage dari Supabase ke Cloudinary
</commit_message>
<xml_diff>
--- a/media/testing jabatan dan departemen.xlsx
+++ b/media/testing jabatan dan departemen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project Pyton\BackUp-HRIS-SMARTDESK -3 - Deploy\media\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFF1CEDF-6992-4658-9434-6E2F5AD088E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2A8ABC6-EBEE-44D8-9662-A91F45103F38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C055B750-2FAD-4A97-A9C6-0F998466A184}"/>
   </bookViews>
@@ -87,346 +87,346 @@
     <t>Human Resources | HR</t>
   </si>
   <si>
-    <t>14. Corporate Management</t>
-  </si>
-  <si>
-    <t>13. Management</t>
-  </si>
-  <si>
-    <t>1. Mining Department , MPE-MIN</t>
-  </si>
-  <si>
-    <t>2. Civil &amp; Maintenance , CIV-MAINT</t>
-  </si>
-  <si>
-    <t>3. Electric &amp; Utility , EWF</t>
-  </si>
-  <si>
-    <t>4. Health Safety Environment , HSE</t>
-  </si>
-  <si>
-    <t>5. Human Resources , HR</t>
-  </si>
-  <si>
-    <t>6. General Affair , GA</t>
-  </si>
-  <si>
-    <t>7. Logistic &amp; Warehouse , LOG</t>
-  </si>
-  <si>
-    <t>8. Purchasing , PURCH</t>
-  </si>
-  <si>
-    <t>9. Finance &amp; Accounting , FAT</t>
-  </si>
-  <si>
-    <t>10. Infrastructure Technology , IT</t>
-  </si>
-  <si>
-    <t>11. Legal , LGL</t>
-  </si>
-  <si>
-    <t>12. Security , SG</t>
-  </si>
-  <si>
-    <t>Operator ADT , Crew , Mining</t>
-  </si>
-  <si>
-    <t>Operator Excavator , Crew , Mining</t>
-  </si>
-  <si>
-    <t>Operator Dozer , Crew , Mining</t>
-  </si>
-  <si>
-    <t>Operator Grader , Crew , Mining</t>
-  </si>
-  <si>
-    <t>Operator Loader , Crew , Mining</t>
-  </si>
-  <si>
-    <t>Surveyor , Staff , Mining</t>
-  </si>
-  <si>
-    <t>Mine Dispatcher , Staff , Mining</t>
-  </si>
-  <si>
-    <t>Drill &amp; Blast Officer , Staff , Mining</t>
-  </si>
-  <si>
-    <t>Mine Engineer , Staff , Mining</t>
-  </si>
-  <si>
-    <t>Senior Mine Engineer , Senior Staff , Mining</t>
-  </si>
-  <si>
-    <t>Mine Foreman , Supervisor , Mining</t>
-  </si>
-  <si>
-    <t>Pit Supervisor , Supervisor , Mining</t>
-  </si>
-  <si>
-    <t>Mining Superintendent , Superintendent , Mining</t>
-  </si>
-  <si>
-    <t>Mine Manager , Manager , Mining</t>
-  </si>
-  <si>
-    <t>Mechanic , Crew , Civil &amp; Maintenance</t>
-  </si>
-  <si>
-    <t>Helper Mechanic , Crew , Civil &amp; Maintenance</t>
-  </si>
-  <si>
-    <t>Welder , Crew , Civil &amp; Maintenance</t>
-  </si>
-  <si>
-    <t>Technician , Staff , Civil &amp; Maintenance</t>
-  </si>
-  <si>
-    <t>Maintenance Planner , Staff , Civil &amp; Maintenance</t>
-  </si>
-  <si>
-    <t>Senior Mechanic , Senior Staff , Civil &amp; Maintenance</t>
-  </si>
-  <si>
-    <t>Foreman Mechanic , Supervisor , Civil &amp; Maintenance</t>
-  </si>
-  <si>
-    <t>Workshop Supervisor , Supervisor , Civil &amp; Maintenance</t>
-  </si>
-  <si>
-    <t>Maintenance Superintendent , Superintendent , Civil &amp; Maintenance</t>
-  </si>
-  <si>
-    <t>Maintenance Manager , Manager , Civil &amp; Maintenance</t>
-  </si>
-  <si>
-    <t>Electrician , Crew , Electric &amp; Water Facility</t>
-  </si>
-  <si>
-    <t>Genset Operator , Crew , Electric &amp; Water Facility</t>
-  </si>
-  <si>
-    <t>Water Pump Operator , Crew , Electric &amp; Water Facility</t>
-  </si>
-  <si>
-    <t>Electrical Technician , Staff , Electric &amp; Water Facility</t>
-  </si>
-  <si>
-    <t>Electrical Engineer , Staff , Electric &amp; Water Facility</t>
-  </si>
-  <si>
-    <t>Senior Electrical Engineer , Senior Staff , Electric &amp; Water Facility</t>
-  </si>
-  <si>
-    <t>Electrical Supervisor , Supervisor , Electric &amp; Water Facility</t>
-  </si>
-  <si>
-    <t>Electrical Superintendent , Superintendent , Electric &amp; Water Facility</t>
-  </si>
-  <si>
-    <t>Utility Manager , Manager , Electric &amp; Water Facility</t>
-  </si>
-  <si>
-    <t>Safety Patrol , Crew , HSE</t>
-  </si>
-  <si>
-    <t>Firefighter , Crew , HSE</t>
-  </si>
-  <si>
-    <t>Safety Officer , Staff , HSE</t>
-  </si>
-  <si>
-    <t>Environmental Officer , Staff , HSE</t>
-  </si>
-  <si>
-    <t>Senior Safety Officer , Senior Staff , HSE</t>
-  </si>
-  <si>
-    <t>Safety Supervisor , Supervisor , HSE</t>
-  </si>
-  <si>
-    <t>HSE Superintendent , Superintendent , HSE</t>
-  </si>
-  <si>
-    <t>HSE Manager , Manager , HSE</t>
-  </si>
-  <si>
-    <t>HR Admin , Staff , HR</t>
-  </si>
-  <si>
-    <t>Recruitment Officer , Staff , HR</t>
-  </si>
-  <si>
-    <t>Training Officer , Staff , HR</t>
-  </si>
-  <si>
-    <t>HR Generalist , Senior Staff , HR</t>
-  </si>
-  <si>
-    <t>HR Supervisor , Supervisor , HR</t>
-  </si>
-  <si>
-    <t>HR Superintendent , Superintendent , HR</t>
-  </si>
-  <si>
-    <t>HR Manager , Manager , HR</t>
-  </si>
-  <si>
-    <t>Office Boy , Crew , GA</t>
-  </si>
-  <si>
-    <t>Office Girl , Crew , GA</t>
-  </si>
-  <si>
-    <t>Driver , Crew , GA</t>
-  </si>
-  <si>
-    <t>Gardener , Crew , GA</t>
-  </si>
-  <si>
-    <t>GA Officer , Staff , GA</t>
-  </si>
-  <si>
-    <t>Mess &amp; Camp Officer , Staff , GA</t>
-  </si>
-  <si>
-    <t>Senior GA Officer , Senior Staff , GA</t>
-  </si>
-  <si>
-    <t>GA Supervisor , Supervisor , GA</t>
-  </si>
-  <si>
-    <t>GA Superintendent , Superintendent , GA</t>
-  </si>
-  <si>
-    <t>GA Manager , Manager , GA</t>
-  </si>
-  <si>
-    <t>Warehouse Helper , Crew , Logistic</t>
-  </si>
-  <si>
-    <t>Storekeeper , Staff , Logistic</t>
-  </si>
-  <si>
-    <t>Logistic Officer , Staff , Logistic</t>
-  </si>
-  <si>
-    <t>Senior Logistic Officer , Senior Staff , Logistic</t>
-  </si>
-  <si>
-    <t>Warehouse Supervisor , Supervisor , Logistic</t>
-  </si>
-  <si>
-    <t>Logistic Superintendent , Superintendent , Logistic</t>
-  </si>
-  <si>
-    <t>Logistic Manager , Manager , Logistic</t>
-  </si>
-  <si>
-    <t>Purchasing Admin , Staff , Purchasing</t>
-  </si>
-  <si>
-    <t>Procurement Officer , Staff , Purchasing</t>
-  </si>
-  <si>
-    <t>Senior Procurement Officer , Senior Staff , Purchasing</t>
-  </si>
-  <si>
-    <t>Procurement Supervisor , Supervisor , Purchasing</t>
-  </si>
-  <si>
-    <t>Procurement Superintendent , Superintendent , Purchasing</t>
-  </si>
-  <si>
-    <t>Procurement Manager , Manager , Purchasing</t>
-  </si>
-  <si>
-    <t>Finance Admin , Staff , Finance</t>
-  </si>
-  <si>
-    <t>Accountant , Staff , Finance</t>
-  </si>
-  <si>
-    <t>Tax Officer , Staff , Finance</t>
-  </si>
-  <si>
-    <t>Senior Accountant , Senior Staff , Finance</t>
-  </si>
-  <si>
-    <t>Finance Supervisor , Supervisor , Finance</t>
-  </si>
-  <si>
-    <t>Finance Superintendent , Superintendent , Finance</t>
-  </si>
-  <si>
-    <t>Finance Manager , Manager , Finance</t>
-  </si>
-  <si>
-    <t>IT Support , Staff , IT</t>
-  </si>
-  <si>
-    <t>Network Engineer , Staff , IT</t>
-  </si>
-  <si>
-    <t>System Administrator , Senior Staff , IT</t>
-  </si>
-  <si>
-    <t>IT Supervisor , Supervisor , IT</t>
-  </si>
-  <si>
-    <t>IT Superintendent , Superintendent , IT</t>
-  </si>
-  <si>
-    <t>IT Manager , Manager , IT</t>
-  </si>
-  <si>
-    <t>Legal Admin , Staff , Legal</t>
-  </si>
-  <si>
-    <t>Legal Officer , Staff , Legal</t>
-  </si>
-  <si>
-    <t>Senior Legal Officer , Senior Staff , Legal</t>
-  </si>
-  <si>
-    <t>Legal Supervisor , Supervisor , Legal</t>
-  </si>
-  <si>
-    <t>Legal Manager , Manager , Legal</t>
-  </si>
-  <si>
-    <t>Security Guard , Crew , Security</t>
-  </si>
-  <si>
-    <t>Security Officer , Staff , Security</t>
-  </si>
-  <si>
-    <t>Senior Security Officer , Senior Staff , Security</t>
-  </si>
-  <si>
-    <t>Security Supervisor , Supervisor , Security</t>
-  </si>
-  <si>
-    <t>Security Manager , Manager , Security</t>
-  </si>
-  <si>
-    <t>Site Superintendent , Superintendent , Site Management</t>
-  </si>
-  <si>
-    <t>Site Manager , Site Manager , Management</t>
-  </si>
-  <si>
-    <t>Operations Director , Director , Corporte Management</t>
-  </si>
-  <si>
-    <t>Finance Director , Director , Corporate Management</t>
-  </si>
-  <si>
-    <t>HR Director , Director , Corporate Management</t>
-  </si>
-  <si>
-    <t>Managing Director , Director , Corporate Management</t>
+    <t>Mining Department,MPE-MIN</t>
+  </si>
+  <si>
+    <t>Civil &amp; Maintenance,CIV-MAINT</t>
+  </si>
+  <si>
+    <t>Electric &amp; Utility,EWF</t>
+  </si>
+  <si>
+    <t>Health Safety Environment,HSE</t>
+  </si>
+  <si>
+    <t>Human Resources,HR</t>
+  </si>
+  <si>
+    <t>General Affair,GA</t>
+  </si>
+  <si>
+    <t>Logistic &amp; Warehouse,LOG</t>
+  </si>
+  <si>
+    <t>Purchasing,PURCH</t>
+  </si>
+  <si>
+    <t>Finance &amp; Accounting,FAT</t>
+  </si>
+  <si>
+    <t>Infrastructure Technology,IT</t>
+  </si>
+  <si>
+    <t>Legal,LGL</t>
+  </si>
+  <si>
+    <t>Security,SG</t>
+  </si>
+  <si>
+    <t>Operator ADT,Crew,Mining</t>
+  </si>
+  <si>
+    <t>Operator Excavator,Crew,Mining</t>
+  </si>
+  <si>
+    <t>Operator Dozer,Crew,Mining</t>
+  </si>
+  <si>
+    <t>Operator Grader,Crew,Mining</t>
+  </si>
+  <si>
+    <t>Operator Loader,Crew,Mining</t>
+  </si>
+  <si>
+    <t>Surveyor,Staff,Mining</t>
+  </si>
+  <si>
+    <t>Mine Dispatcher,Staff,Mining</t>
+  </si>
+  <si>
+    <t>Drill &amp; Blast Officer,Staff,Mining</t>
+  </si>
+  <si>
+    <t>Mine Engineer,Staff,Mining</t>
+  </si>
+  <si>
+    <t>Senior Mine Engineer,Senior Staff,Mining</t>
+  </si>
+  <si>
+    <t>Mine Foreman,Supervisor,Mining</t>
+  </si>
+  <si>
+    <t>Pit Supervisor,Supervisor,Mining</t>
+  </si>
+  <si>
+    <t>Mining Superintendent,Superintendent,Mining</t>
+  </si>
+  <si>
+    <t>Mine Manager,Manager,Mining</t>
+  </si>
+  <si>
+    <t>Mechanic,Crew,Civil &amp; Maintenance</t>
+  </si>
+  <si>
+    <t>Helper Mechanic,Crew,Civil &amp; Maintenance</t>
+  </si>
+  <si>
+    <t>Welder,Crew,Civil &amp; Maintenance</t>
+  </si>
+  <si>
+    <t>Technician,Staff,Civil &amp; Maintenance</t>
+  </si>
+  <si>
+    <t>Maintenance Planner,Staff,Civil &amp; Maintenance</t>
+  </si>
+  <si>
+    <t>Senior Mechanic,Senior Staff,Civil &amp; Maintenance</t>
+  </si>
+  <si>
+    <t>Foreman Mechanic,Supervisor,Civil &amp; Maintenance</t>
+  </si>
+  <si>
+    <t>Workshop Supervisor,Supervisor,Civil &amp; Maintenance</t>
+  </si>
+  <si>
+    <t>Maintenance Superintendent,Superintendent,Civil &amp; Maintenance</t>
+  </si>
+  <si>
+    <t>Maintenance Manager,Manager,Civil &amp; Maintenance</t>
+  </si>
+  <si>
+    <t>Electrician,Crew,Electric &amp; Water Facility</t>
+  </si>
+  <si>
+    <t>Genset Operator,Crew,Electric &amp; Water Facility</t>
+  </si>
+  <si>
+    <t>Water Pump Operator,Crew,Electric &amp; Water Facility</t>
+  </si>
+  <si>
+    <t>Electrical Technician,Staff,Electric &amp; Water Facility</t>
+  </si>
+  <si>
+    <t>Electrical Engineer,Staff,Electric &amp; Water Facility</t>
+  </si>
+  <si>
+    <t>Senior Electrical Engineer,Senior Staff,Electric &amp; Water Facility</t>
+  </si>
+  <si>
+    <t>Electrical Supervisor,Supervisor,Electric &amp; Water Facility</t>
+  </si>
+  <si>
+    <t>Electrical Superintendent,Superintendent,Electric &amp; Water Facility</t>
+  </si>
+  <si>
+    <t>Utility Manager,Manager,Electric &amp; Water Facility</t>
+  </si>
+  <si>
+    <t>Safety Patrol,Crew,HSE</t>
+  </si>
+  <si>
+    <t>Firefighter,Crew,HSE</t>
+  </si>
+  <si>
+    <t>Safety Officer,Staff,HSE</t>
+  </si>
+  <si>
+    <t>Environmental Officer,Staff,HSE</t>
+  </si>
+  <si>
+    <t>Senior Safety Officer,Senior Staff,HSE</t>
+  </si>
+  <si>
+    <t>Safety Supervisor,Supervisor,HSE</t>
+  </si>
+  <si>
+    <t>HSE Superintendent,Superintendent,HSE</t>
+  </si>
+  <si>
+    <t>HSE Manager,Manager,HSE</t>
+  </si>
+  <si>
+    <t>HR Admin,Staff,HR</t>
+  </si>
+  <si>
+    <t>Recruitment Officer,Staff,HR</t>
+  </si>
+  <si>
+    <t>Training Officer,Staff,HR</t>
+  </si>
+  <si>
+    <t>HR Generalist,Senior Staff,HR</t>
+  </si>
+  <si>
+    <t>HR Supervisor,Supervisor,HR</t>
+  </si>
+  <si>
+    <t>HR Superintendent,Superintendent,HR</t>
+  </si>
+  <si>
+    <t>HR Manager,Manager,HR</t>
+  </si>
+  <si>
+    <t>Office Boy,Crew,GA</t>
+  </si>
+  <si>
+    <t>Office Girl,Crew,GA</t>
+  </si>
+  <si>
+    <t>Driver,Crew,GA</t>
+  </si>
+  <si>
+    <t>Gardener,Crew,GA</t>
+  </si>
+  <si>
+    <t>GA Officer,Staff,GA</t>
+  </si>
+  <si>
+    <t>Mess &amp; Camp Officer,Staff,GA</t>
+  </si>
+  <si>
+    <t>Senior GA Officer,Senior Staff,GA</t>
+  </si>
+  <si>
+    <t>GA Supervisor,Supervisor,GA</t>
+  </si>
+  <si>
+    <t>GA Superintendent,Superintendent,GA</t>
+  </si>
+  <si>
+    <t>GA Manager,Manager,GA</t>
+  </si>
+  <si>
+    <t>Warehouse Helper,Crew,Logistic</t>
+  </si>
+  <si>
+    <t>Storekeeper,Staff,Logistic</t>
+  </si>
+  <si>
+    <t>Logistic Officer,Staff,Logistic</t>
+  </si>
+  <si>
+    <t>Senior Logistic Officer,Senior Staff,Logistic</t>
+  </si>
+  <si>
+    <t>Warehouse Supervisor,Supervisor,Logistic</t>
+  </si>
+  <si>
+    <t>Logistic Superintendent,Superintendent,Logistic</t>
+  </si>
+  <si>
+    <t>Logistic Manager,Manager,Logistic</t>
+  </si>
+  <si>
+    <t>Purchasing Admin,Staff,Purchasing</t>
+  </si>
+  <si>
+    <t>Procurement Officer,Staff,Purchasing</t>
+  </si>
+  <si>
+    <t>Senior Procurement Officer,Senior Staff,Purchasing</t>
+  </si>
+  <si>
+    <t>Procurement Supervisor,Supervisor,Purchasing</t>
+  </si>
+  <si>
+    <t>Procurement Superintendent,Superintendent,Purchasing</t>
+  </si>
+  <si>
+    <t>Procurement Manager,Manager,Purchasing</t>
+  </si>
+  <si>
+    <t>Finance Admin,Staff,Finance</t>
+  </si>
+  <si>
+    <t>Accountant,Staff,Finance</t>
+  </si>
+  <si>
+    <t>Tax Officer,Staff,Finance</t>
+  </si>
+  <si>
+    <t>Senior Accountant,Senior Staff,Finance</t>
+  </si>
+  <si>
+    <t>Finance Supervisor,Supervisor,Finance</t>
+  </si>
+  <si>
+    <t>Finance Superintendent,Superintendent,Finance</t>
+  </si>
+  <si>
+    <t>Finance Manager,Manager,Finance</t>
+  </si>
+  <si>
+    <t>IT Support,Staff,IT</t>
+  </si>
+  <si>
+    <t>Network Engineer,Staff,IT</t>
+  </si>
+  <si>
+    <t>System Administrator,Senior Staff,IT</t>
+  </si>
+  <si>
+    <t>IT Supervisor,Supervisor,IT</t>
+  </si>
+  <si>
+    <t>IT Superintendent,Superintendent,IT</t>
+  </si>
+  <si>
+    <t>IT Manager,Manager,IT</t>
+  </si>
+  <si>
+    <t>Legal Admin,Staff,Legal</t>
+  </si>
+  <si>
+    <t>Legal Officer,Staff,Legal</t>
+  </si>
+  <si>
+    <t>Senior Legal Officer,Senior Staff,Legal</t>
+  </si>
+  <si>
+    <t>Legal Supervisor,Supervisor,Legal</t>
+  </si>
+  <si>
+    <t>Legal Manager,Manager,Legal</t>
+  </si>
+  <si>
+    <t>Security Guard,Crew,Security</t>
+  </si>
+  <si>
+    <t>Security Officer,Staff,Security</t>
+  </si>
+  <si>
+    <t>Senior Security Officer,Senior Staff,Security</t>
+  </si>
+  <si>
+    <t>Security Supervisor,Supervisor,Security</t>
+  </si>
+  <si>
+    <t>Security Manager,Manager,Security</t>
+  </si>
+  <si>
+    <t>Site Superintendent,Superintendent,Site Management</t>
+  </si>
+  <si>
+    <t>Site Manager,Site Manager,Management</t>
+  </si>
+  <si>
+    <t>Operations Director,Director,Corporte Management</t>
+  </si>
+  <si>
+    <t>Finance Director,Director,Corporate Management</t>
+  </si>
+  <si>
+    <t>HR Director,Director,Corporate Management</t>
+  </si>
+  <si>
+    <t>Managing Director,Director,Corporate Management</t>
+  </si>
+  <si>
+    <t>Management,MGM</t>
+  </si>
+  <si>
+    <t>Corporate Management,CMGM</t>
   </si>
 </sst>
 </file>
@@ -841,7 +841,7 @@
         <v>0</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -849,7 +849,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -857,7 +857,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -865,7 +865,7 @@
         <v>3</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -873,7 +873,7 @@
         <v>4</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -881,7 +881,7 @@
         <v>5</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -889,7 +889,7 @@
         <v>16</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -897,7 +897,7 @@
         <v>6</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -905,7 +905,7 @@
         <v>7</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -913,7 +913,7 @@
         <v>8</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -921,7 +921,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -929,7 +929,7 @@
         <v>10</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -937,7 +937,7 @@
         <v>11</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>18</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -945,7 +945,7 @@
         <v>12</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>17</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -953,7 +953,7 @@
         <v>13</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -961,7 +961,7 @@
         <v>14</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -969,492 +969,492 @@
         <v>15</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E18" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E19" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E20" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E21" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E22" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E23" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E24" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E25" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E26" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E27" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E28" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E29" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E30" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E31" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E32" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="33" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E33" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="34" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E34" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E35" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="36" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E36" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="37" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E37" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="38" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E38" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="39" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E39" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="40" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E40" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="41" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E41" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="42" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E42" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="43" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E43" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="44" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E44" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="45" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E45" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="46" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E46" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="47" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E47" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="48" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E48" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E49" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E50" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E51" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E52" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E53" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E54" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E55" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E56" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E57" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="58" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E58" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="59" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E59" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="60" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E60" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="61" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E61" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="62" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E62" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="63" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E63" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="64" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E64" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="65" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E65" s="5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="66" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E66" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="67" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E67" s="5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="68" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E68" s="5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="69" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E69" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="70" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E70" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="71" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E71" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="72" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E72" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="73" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E73" s="5" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="74" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E74" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="75" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E75" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="76" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E76" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="77" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E77" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="78" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E78" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="79" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E79" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="80" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E80" s="5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="81" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E81" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="82" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E82" s="5" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="83" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E83" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="84" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E84" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="85" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E85" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="86" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E86" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="87" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E87" s="5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="88" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E88" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="89" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E89" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="90" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E90" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="91" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E91" s="5" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="92" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E92" s="5" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="93" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E93" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="94" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E94" s="5" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="95" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E95" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="96" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E96" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="97" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E97" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="98" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E98" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="99" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E99" s="5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="100" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E100" s="5" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="101" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E101" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="102" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E102" s="5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="103" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E103" s="5" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="104" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E104" s="5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="105" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E105" s="5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="106" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E106" s="5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="107" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E107" s="5" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="108" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E108" s="5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="109" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E109" s="5" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="110" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E110" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="111" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E111" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="112" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E112" s="5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="113" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E113" s="5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="114" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E114" s="5" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>